<commit_message>
Import B2 sales 1-17 Oct 2026 from Parn's photos (approved by Parn)
17 days, revenue 63,924 (before ice), expenses (ice) 1,110. Oct26 sheet moved to the Sep26 column layout. 13 Oct sheet says B-1; Parn confirmed B2.
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B2_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B2_2026.xlsx
@@ -136,10 +136,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -171,10 +171,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -3712,7 +3712,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:AF20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3745,39 +3745,883 @@
         <v>Orange</v>
       </c>
       <c r="I3" t="str">
+        <v>Orange (100)</v>
+      </c>
+      <c r="J3" t="str">
         <v>Watermelon</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>Mango</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>Coconut</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>Apple</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>Young Coco</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
+        <v>Guava</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Pineapple</v>
+      </c>
+      <c r="Q3" t="str">
         <v>Total Cups</v>
       </c>
-      <c r="O3" t="str">
+      <c r="R3" t="str">
         <v>Bot Big</v>
       </c>
-      <c r="P3" t="str">
+      <c r="S3" t="str">
         <v>Bot Small</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="T3" t="str">
         <v>Used Orange (basket)</v>
       </c>
-      <c r="R3" t="str">
+      <c r="U3" t="str">
         <v>Used Watermelon (pcs)</v>
+      </c>
+      <c r="V3" t="str">
+        <v>Used Mango</v>
+      </c>
+      <c r="W3" t="str">
+        <v>Used Coco (Meat)</v>
+      </c>
+      <c r="X3" t="str">
+        <v>Used Coco (Water)</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>Used Coco (Conden)</v>
+      </c>
+      <c r="Z3" t="str">
+        <v>Used Coco (Raw)</v>
+      </c>
+      <c r="AA3" t="str">
+        <v>Used Apple</v>
+      </c>
+      <c r="AB3" t="str">
+        <v>Used Guava</v>
+      </c>
+      <c r="AC3" t="str">
+        <v>Used Pineapple</v>
+      </c>
+      <c r="AD3" t="str">
+        <v>Used Young Coco</v>
+      </c>
+      <c r="AE3" t="str">
+        <v>Bottle Revenue (฿)</v>
+      </c>
+      <c r="AF3" t="str">
+        <v>Source Note</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C4">
+        <v>2699</v>
+      </c>
+      <c r="D4">
+        <v>1890</v>
+      </c>
+      <c r="E4">
+        <v>60</v>
+      </c>
+      <c r="G4">
+        <v>809</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>12</v>
+      </c>
+      <c r="K4">
+        <v>4</v>
+      </c>
+      <c r="L4">
+        <v>9</v>
+      </c>
+      <c r="M4">
+        <v>10</v>
+      </c>
+      <c r="O4">
+        <v>3</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>40</v>
+      </c>
+      <c r="AF4" t="str">
+        <v>Parn LINE photo 01M56Z0ZBJM60G0S61HHCMW2DT.jpg (B2 Daily Sales Record 01/10/26), hand-transcribed 2026-10-18 | sheet totals are after ice (cash 1830, grand 2639); booked before ice, ice in Expenses like B1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C5">
+        <v>3364</v>
+      </c>
+      <c r="D5">
+        <v>2090</v>
+      </c>
+      <c r="E5">
+        <v>60</v>
+      </c>
+      <c r="G5">
+        <v>1274</v>
+      </c>
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <v>14</v>
+      </c>
+      <c r="K5">
+        <v>3</v>
+      </c>
+      <c r="L5">
+        <v>20</v>
+      </c>
+      <c r="M5">
+        <v>3</v>
+      </c>
+      <c r="O5">
+        <v>4</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>51</v>
+      </c>
+      <c r="AF5" t="str">
+        <v>Parn LINE photo 01M56Z15SBMB2AJ72MF67WNAFF.jpg (B2 Daily Sales Record 02/10/26), hand-transcribed 2026-10-18 | sheet totals are after ice (cash 2030, grand 3304); booked before ice, ice in Expenses like B1 | CHECK: QR items 1,334 vs written 1,274 (+60)</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>03/10/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C6">
+        <v>4304</v>
+      </c>
+      <c r="D6">
+        <v>2699</v>
+      </c>
+      <c r="E6">
+        <v>60</v>
+      </c>
+      <c r="G6">
+        <v>1605</v>
+      </c>
+      <c r="H6">
+        <v>7</v>
+      </c>
+      <c r="J6">
+        <v>20</v>
+      </c>
+      <c r="K6">
+        <v>3</v>
+      </c>
+      <c r="L6">
+        <v>9</v>
+      </c>
+      <c r="M6">
+        <v>5</v>
+      </c>
+      <c r="O6">
+        <v>8</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>60</v>
+      </c>
+      <c r="AF6" t="str">
+        <v>Parn LINE photo 01M56Z15M9VGJBP7BYXAYEMHN7.jpg (B2 Daily Sales Record 03/10/26), hand-transcribed 2026-10-18 | sheet totals are after ice (cash 2639, grand 4244); booked before ice, ice in Expenses like B1 | not in fruit columns: Grape 1, Pear 2, Pomegranate 5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>04/10/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C7">
+        <v>3608</v>
+      </c>
+      <c r="D7">
+        <v>2263</v>
+      </c>
+      <c r="E7">
+        <v>60</v>
+      </c>
+      <c r="G7">
+        <v>1345</v>
+      </c>
+      <c r="H7">
+        <v>8</v>
+      </c>
+      <c r="J7">
+        <v>17</v>
+      </c>
+      <c r="K7">
+        <v>4</v>
+      </c>
+      <c r="L7">
+        <v>8</v>
+      </c>
+      <c r="M7">
+        <v>3</v>
+      </c>
+      <c r="O7">
+        <v>3</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>50</v>
+      </c>
+      <c r="AF7" t="str">
+        <v>Parn LINE photo 01M56Z15FGPG5BS25GHH9YM5NC.jpg (B2 Daily Sales Record 04/10/26), hand-transcribed 2026-10-18 | sheet totals are after ice (cash 2203, grand 3548); booked before ice, ice in Expenses like B1 | not in fruit columns: Pomegranate 2, Grape 1, Grape (120) 1, Pear 3 | CHECK: cash items 2,253 vs written 2,263 (-10)</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>05/10/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C8">
+        <v>2775</v>
+      </c>
+      <c r="D8">
+        <v>1890</v>
+      </c>
+      <c r="E8">
+        <v>60</v>
+      </c>
+      <c r="G8">
+        <v>885</v>
+      </c>
+      <c r="H8">
+        <v>9</v>
+      </c>
+      <c r="J8">
+        <v>13</v>
+      </c>
+      <c r="K8">
+        <v>5</v>
+      </c>
+      <c r="L8">
+        <v>5</v>
+      </c>
+      <c r="M8">
+        <v>4</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>40</v>
+      </c>
+      <c r="AF8" t="str">
+        <v>Parn LINE photo 01M56Z14Z0PDC1NC3BPYD52JAT.jpg (B2 Daily Sales Record 05/10/26), hand-transcribed 2026-10-18 | sheet totals are after ice (cash 1830, grand 2715); booked before ice, ice in Expenses like B1 | not in fruit columns: Pear 2, Grape 1, Pomegranate 1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>06/10/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C9">
+        <v>2234</v>
+      </c>
+      <c r="D9">
+        <v>1529</v>
+      </c>
+      <c r="E9">
+        <v>60</v>
+      </c>
+      <c r="G9">
+        <v>705</v>
+      </c>
+      <c r="H9">
+        <v>3</v>
+      </c>
+      <c r="J9">
+        <v>12</v>
+      </c>
+      <c r="K9">
+        <v>3</v>
+      </c>
+      <c r="L9">
+        <v>4</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>2</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>30</v>
+      </c>
+      <c r="AF9" t="str">
+        <v>Parn LINE photo 01M56Z14T0V8CC9DFHRS56D9PQ.jpg (B2 Daily Sales Record 06/10/26), hand-transcribed 2026-10-18 | sheet totals are after ice (cash 1469, grand 2174); booked before ice, ice in Expenses like B1 | not in fruit columns: Pear 3, Pomegranate 3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>07/10/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C10">
+        <v>2605</v>
+      </c>
+      <c r="D10">
+        <v>1525</v>
+      </c>
+      <c r="E10">
+        <v>60</v>
+      </c>
+      <c r="G10">
+        <v>1080</v>
+      </c>
+      <c r="H10">
+        <v>5</v>
+      </c>
+      <c r="J10">
+        <v>11</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>12</v>
+      </c>
+      <c r="M10">
+        <v>5</v>
+      </c>
+      <c r="O10">
+        <v>2</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>38</v>
+      </c>
+      <c r="AF10" t="str">
+        <v>Parn LINE photo 01M56Z1446RJT12Q7FSDJR407H.jpg (B2 Daily Sales Record 07/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>08/10/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C11">
+        <v>2080</v>
+      </c>
+      <c r="D11">
+        <v>1115</v>
+      </c>
+      <c r="E11">
+        <v>60</v>
+      </c>
+      <c r="G11">
+        <v>965</v>
+      </c>
+      <c r="H11">
+        <v>6</v>
+      </c>
+      <c r="J11">
+        <v>10</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>2</v>
+      </c>
+      <c r="M11">
+        <v>6</v>
+      </c>
+      <c r="O11">
+        <v>6</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>33</v>
+      </c>
+      <c r="AF11" t="str">
+        <v>Parn LINE photo 01M56Z14SM75C5WBM25A8RMMS8.jpg (B2 Daily Sales Record 08/10/26), hand-transcribed 2026-10-18 | sheet totals are after ice (cash 1055, grand 2020); booked before ice, ice in Expenses like B1 | not in fruit columns: Pear 3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C12">
+        <v>3200</v>
+      </c>
+      <c r="D12">
+        <v>2730</v>
+      </c>
+      <c r="E12">
+        <v>60</v>
+      </c>
+      <c r="G12">
+        <v>470</v>
+      </c>
+      <c r="H12">
+        <v>5</v>
+      </c>
+      <c r="J12">
+        <v>11</v>
+      </c>
+      <c r="K12">
+        <v>1</v>
+      </c>
+      <c r="L12">
+        <v>11</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
+      </c>
+      <c r="O12">
+        <v>1</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>40</v>
+      </c>
+      <c r="AF12" t="str">
+        <v>Parn LINE photo 01M56Z141JFX6801S3WJCTH01P.jpg (B2 Daily Sales Record 09/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 8, Pear 2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>10/10/2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C13">
+        <v>7064</v>
+      </c>
+      <c r="D13">
+        <v>4759</v>
+      </c>
+      <c r="E13">
+        <v>90</v>
+      </c>
+      <c r="G13">
+        <v>2305</v>
+      </c>
+      <c r="H13">
+        <v>9</v>
+      </c>
+      <c r="J13">
+        <v>33</v>
+      </c>
+      <c r="K13">
+        <v>10</v>
+      </c>
+      <c r="L13">
+        <v>18</v>
+      </c>
+      <c r="M13">
+        <v>4</v>
+      </c>
+      <c r="O13">
+        <v>5</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>96</v>
+      </c>
+      <c r="AF13" t="str">
+        <v>Parn LINE photo 01M56Z0ZC83MFZ6E6E3AN602KM.jpg (B2 Daily Sales Record 10/10/26), hand-transcribed 2026-10-18 | sheet totals are after ice (cash 4669, grand 6974); booked before ice, ice in Expenses like B1 | not in fruit columns: Pomegranate 10, Pear 7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>11/10/2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C14">
+        <v>6005</v>
+      </c>
+      <c r="D14">
+        <v>4625</v>
+      </c>
+      <c r="E14">
+        <v>60</v>
+      </c>
+      <c r="G14">
+        <v>1380</v>
+      </c>
+      <c r="H14">
+        <v>8</v>
+      </c>
+      <c r="J14">
+        <v>26</v>
+      </c>
+      <c r="K14">
+        <v>9</v>
+      </c>
+      <c r="L14">
+        <v>7</v>
+      </c>
+      <c r="M14">
+        <v>15</v>
+      </c>
+      <c r="O14">
+        <v>7</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>81</v>
+      </c>
+      <c r="AF14" t="str">
+        <v>Parn LINE photo 01M56Z10B45G5BY8KB6VNWF1BG.jpg (B2 Daily Sales Record 11/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C15">
+        <v>6260</v>
+      </c>
+      <c r="D15">
+        <v>4050</v>
+      </c>
+      <c r="E15">
+        <v>120</v>
+      </c>
+      <c r="G15">
+        <v>2210</v>
+      </c>
+      <c r="H15">
+        <v>13</v>
+      </c>
+      <c r="J15">
+        <v>39</v>
+      </c>
+      <c r="K15">
+        <v>3</v>
+      </c>
+      <c r="L15">
+        <v>14</v>
+      </c>
+      <c r="M15">
+        <v>13</v>
+      </c>
+      <c r="O15">
+        <v>9</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>95</v>
+      </c>
+      <c r="AF15" t="str">
+        <v>Parn LINE photo 01M56Z12TMRXN4ANPV2TGN9Z5B.jpg (B2 Daily Sales Record 12/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>13/10/2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C16">
+        <v>4019</v>
+      </c>
+      <c r="D16">
+        <v>1984</v>
+      </c>
+      <c r="E16">
+        <v>60</v>
+      </c>
+      <c r="G16">
+        <v>2035</v>
+      </c>
+      <c r="H16">
+        <v>8</v>
+      </c>
+      <c r="J16">
+        <v>13</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>10</v>
+      </c>
+      <c r="M16">
+        <v>14</v>
+      </c>
+      <c r="O16">
+        <v>4</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>55</v>
+      </c>
+      <c r="AF16" t="str">
+        <v>Parn LINE photo 01M56Z0ZDFSRGCG6GRCTYJAE97.jpg (B2 Daily Sales Record 13/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>14/10/2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C17">
+        <v>2485</v>
+      </c>
+      <c r="D17">
+        <v>1690</v>
+      </c>
+      <c r="E17">
+        <v>60</v>
+      </c>
+      <c r="G17">
+        <v>795</v>
+      </c>
+      <c r="H17">
+        <v>2</v>
+      </c>
+      <c r="J17">
+        <v>12</v>
+      </c>
+      <c r="K17">
+        <v>4</v>
+      </c>
+      <c r="L17">
+        <v>7</v>
+      </c>
+      <c r="M17">
+        <v>4</v>
+      </c>
+      <c r="O17">
+        <v>3</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>35</v>
+      </c>
+      <c r="AF17" t="str">
+        <v>Parn LINE photo 01M56Z0ZB74KJXCFW22ZCM69CA.jpg (B2 Daily Sales Record 14/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>15/10/2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C18">
+        <v>3630</v>
+      </c>
+      <c r="D18">
+        <v>1937</v>
+      </c>
+      <c r="E18">
+        <v>60</v>
+      </c>
+      <c r="G18">
+        <v>1693</v>
+      </c>
+      <c r="H18">
+        <v>8</v>
+      </c>
+      <c r="J18">
+        <v>14</v>
+      </c>
+      <c r="K18">
+        <v>2</v>
+      </c>
+      <c r="L18">
+        <v>5</v>
+      </c>
+      <c r="M18">
+        <v>5</v>
+      </c>
+      <c r="O18">
+        <v>8</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+      <c r="Q18">
+        <v>46</v>
+      </c>
+      <c r="AF18" t="str">
+        <v>Parn LINE photo 01M56Z10C2KT4J7NZNFGB0HRX1.jpg (B2 Daily Sales Record 15/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>16/10/2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C19">
+        <v>4058</v>
+      </c>
+      <c r="D19">
+        <v>2743</v>
+      </c>
+      <c r="E19">
+        <v>60</v>
+      </c>
+      <c r="G19">
+        <v>1315</v>
+      </c>
+      <c r="H19">
+        <v>8</v>
+      </c>
+      <c r="J19">
+        <v>20</v>
+      </c>
+      <c r="K19">
+        <v>7</v>
+      </c>
+      <c r="L19">
+        <v>10</v>
+      </c>
+      <c r="M19">
+        <v>2</v>
+      </c>
+      <c r="O19">
+        <v>6</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>56</v>
+      </c>
+      <c r="AF19" t="str">
+        <v>Parn LINE photo 01M56Z123JEEQQNSJGBRPBB9CP.jpg (B2 Daily Sales Record 16/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>17/10/2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C20">
+        <v>3534</v>
+      </c>
+      <c r="D20">
+        <v>1639</v>
+      </c>
+      <c r="E20">
+        <v>60</v>
+      </c>
+      <c r="G20">
+        <v>1895</v>
+      </c>
+      <c r="H20">
+        <v>5</v>
+      </c>
+      <c r="J20">
+        <v>18</v>
+      </c>
+      <c r="K20">
+        <v>3</v>
+      </c>
+      <c r="L20">
+        <v>7</v>
+      </c>
+      <c r="M20">
+        <v>7</v>
+      </c>
+      <c r="O20">
+        <v>8</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>51</v>
+      </c>
+      <c r="AF20" t="str">
+        <v>Parn LINE photo 01M56Z13TMVJBJY5H88SYRP0CP.jpg (B2 Daily Sales Record 17/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 3</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>